<commit_message>
Check complete with confidential files present
</commit_message>
<xml_diff>
--- a/_readme/figure-mapping.xlsx
+++ b/_readme/figure-mapping.xlsx
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
+  <si>
+    <t xml:space="preserve">Appendix</t>
+  </si>
   <si>
     <t xml:space="preserve">Figure number</t>
   </si>
@@ -34,6 +37,9 @@
     <t xml:space="preserve">Program</t>
   </si>
   <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
     <t xml:space="preserve">figure1.png</t>
   </si>
   <si>
@@ -58,7 +64,7 @@
     <t xml:space="preserve">fig:software</t>
   </si>
   <si>
-    <t xml:space="preserve">Obtained from Vilhuber (2022a)</t>
+    <t xml:space="preserve">Obtained from Vilhuber (2020a)</t>
   </si>
   <si>
     <t xml:space="preserve">outputs/compare_combined_diff_select.png</t>
@@ -101,6 +107,9 @@
   </si>
   <si>
     <t xml:space="preserve">data/christensen-2019-fig7-legend.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
   </si>
   <si>
     <t xml:space="preserve">6a</t>
@@ -199,7 +208,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -326,19 +335,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D1048576"/>
-  <sheetFormatPr defaultColWidth="11.47265625" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultColWidth="11.47265625" defaultRowHeight="12.65" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="44.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="3.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="44.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="3.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.65"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -350,203 +360,180 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="D5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="A6" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="22.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="2" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>31</v>
+      <c r="B11" s="1" t="s">
+        <v>33</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="1048521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048528" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048529" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048537" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048538" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048541" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048542" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048546" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048547" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048548" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048549" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048550" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048551" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048552" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>34</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>